<commit_message>
feat: incluido uma coluna de decisao do LLM para cada resultado nas planilhas de revisão
</commit_message>
<xml_diff>
--- a/data/review/gpt-5.4-pro/step-3-review.xlsx
+++ b/data/review/gpt-5.4-pro/step-3-review.xlsx
@@ -420,13 +420,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D340"/>
+  <dimension ref="A1:E340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="90" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,6 +448,11 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>llm_decision</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>decision</t>
         </is>
       </c>
@@ -467,7 +473,12 @@
           <t>Code generation, Code repair, Large language models, Static analysis</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -485,7 +496,12 @@
           <t>Code refactoring, Consistency, Empirical study, large language models, Prompt</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -503,7 +519,12 @@
           <t>Cangjie, code completion, cross-language knowledge, Large Language Models (LLMs), low-resource programming languages, transfer learning</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -521,7 +542,12 @@
           <t>AI in software refactoring, Artificial Intelligence, Data augmentation, LLMs in software engineering, Machine learning, Refactoring</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -539,7 +565,12 @@
           <t>Large language models, LLVM IR, Neural decompilation, Symbolic execution</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -557,7 +588,12 @@
           <t>AI augmented software engineering, LLM, Multi agent, Scrum, Sprint</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -575,7 +611,12 @@
           <t>API contract, Codebase, Coding rules, Source code generation, UI design, Use case specification, Vibe coding, Website generation</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -593,7 +634,12 @@
           <t>Class diagrams generation, Model-driven development, NLP transformer, Requirement analysis</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -611,7 +657,12 @@
           <t>Fine-tuning, GoF patterns, LLMs, Seq2Seq models, Software engineering, Transformer architecture</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -629,7 +680,12 @@
           <t>Artificial intelligence, Large language models, Refactoring, Software engineering, Software quality</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -647,7 +703,12 @@
           <t>AI-generated code, Authorship attribution, Code watermarking, Large language models, Software provenance, Systematic literature review</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -665,7 +726,12 @@
           <t>Design patterns, GenAI, Quality, SOLID principles</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -683,7 +749,12 @@
           <t>Code generation, LLM-generated code, Maintainability, Non-functional quality characteristics, Performance efficiency, Security</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -701,7 +772,12 @@
           <t>Bug fixing, Large Language Model, LLM cost analysis, Software development history</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -719,7 +795,12 @@
           <t>Benchmarks, Code generation, Empirical study, Generative AI, Small language models, Software engineering</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -737,7 +818,12 @@
           <t>Code generation, Information retrieval, Large language models, Retrieval-augmented generation</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -755,7 +841,12 @@
           <t>Code instruction tuning, Code intelligence, Large language models, Post-training, Structural pruning</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -773,7 +864,12 @@
           <t>Efficient code generation, large language model (LLM), reinforcement learning (RL)</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -787,7 +883,12 @@
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -805,7 +906,12 @@
           <t>agent-based design, artificial intelligence, autonomous agents, conceptual design, context management, design automation, engineering design, human–AI collaboration, large language models, multi-agent systems, systems design, systems engineering</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -823,7 +929,12 @@
           <t>artificial intelligence, code generation, extended finite state machine, large language models, requirements engineering, software engineering, test automation</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -841,7 +952,12 @@
           <t>AI-assisted programming, Empirical study, Generative AI, Non-programmers, Software engineering</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -859,7 +975,12 @@
           <t>Code Generation, Large Language Models, Mutant Generation, Survived Mutants, Test Suite Augmentation</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -877,7 +998,12 @@
           <t>code generation, code security, evaluation methodology, large language models, neural code intelligence, program synthesis, software engineering</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -895,7 +1021,12 @@
           <t>GenAI, Generative artificial intelligence, Large language model, LLM, Metric, Quality evaluation</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -913,7 +1044,12 @@
           <t>ChatGPT, Code clone, Refactoring, Software quality</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -931,7 +1067,12 @@
           <t>Generative artificial intelligence, Incident management, Software asset management, Software ecosystems, Software quality</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -949,7 +1090,12 @@
           <t>automated software engineering, code generation, direct preference optimization, Large language models, LLM-as-a-Judge, reinforcement learning from AI feedback</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -967,7 +1113,12 @@
           <t>Business models framework, Energy communities, Large language models, Local energy markets, Template-driven code generation</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -985,7 +1136,12 @@
           <t>Additional Key Words and Phrases: Language models for Code, Code generation, Code intelligence, Software engineering, Trustworthiness</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1003,7 +1159,12 @@
           <t>Code Identifier, Evaluation of Tools, Natural Language Processing, Part-of-speech Tagging</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1021,7 +1182,12 @@
           <t>artificial intelligence (AI), empirical software engineering, explainable AI, mobile development, software engineering</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1039,7 +1205,12 @@
           <t>Code Generation, DocString Compression, Large Language Model</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1057,7 +1228,12 @@
           <t>code generation, Halstead complexity, large language models, linguistic similarity, LLM applications, summarization</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1075,7 +1251,12 @@
           <t>large language models, LLM comparison, retrieval-augmented generation, Vulnerability detection</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1093,7 +1274,12 @@
           <t>interactive agents, Large language models, multi-agent systems, software artifact quality, software engineering automation</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1111,7 +1297,12 @@
           <t>generative artificial intelligence, Intent-based-networks, large language models</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1129,7 +1320,12 @@
           <t>ChatGPT, Coding, Large Language Models, Programming Languages, Software Engineering</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1147,7 +1343,12 @@
           <t>API misuse, automatic program repair, Code generation, empirical software engineering, large language model</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1162,7 +1363,12 @@
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1180,7 +1386,12 @@
           <t>Collaboration, educational data mining, feature extraction, Git, large language models, software engineering education, version control mining</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1198,7 +1409,12 @@
           <t>Benchmarks, Code Generation, Empirical Study, Large Language Models for Code</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1216,7 +1432,12 @@
           <t>AI-assisted software engineering, AI-driven software refactoring legacy systems modernization, architecture reconstruction, domain layer reconstruction, GPT, Keywords—Domain-Driven Design, large language models, LLM, semantic code analysis</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1234,7 +1455,12 @@
           <t>Code generation, hallucination, large language models</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1252,7 +1478,12 @@
           <t>code generation, end-to-end software development, Generative artificial intelligence (GenAI), large language models (LLMs), RUPPs templates, sequence diagram generation, structured natural language (SNL), UML class diagram generation, verification and optimization, VeriGen tool</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1266,7 +1497,12 @@
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1284,7 +1520,12 @@
           <t>AI-generated code, code comprehension, institutional knowledge, large language models, software maintenance, technical debt</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1302,7 +1543,12 @@
           <t>large language model (LLM), retrieval-augmented generation (RAG), software engineering, 大语言模型, 检索增强生成, 软件工程</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1320,7 +1566,12 @@
           <t>ChatGPT, generative AI, object oriented, prompt engineering, refactoring</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1338,7 +1589,12 @@
           <t>abstract syntax tree, automated software engineering, code generation, neural networks</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1356,7 +1612,12 @@
           <t>Automatic annotating, autonomous driving, multimodal data annotation, natural language to code generation</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1374,7 +1635,12 @@
           <t>AI-drivenrefactoring, Artificial intelligence, code-level refactoring, CodeSearchNet, CQRS, legacy systems, command and query responsibility segregation, LLM, software architecture refactoring, software engineering</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1392,7 +1658,12 @@
           <t>code bias, interpretability bias, Large language models, security implications, software engineering</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1410,7 +1681,12 @@
           <t>Assessment, Code refactoring, Design patterns, Large language models (LLMs), Metrics, Pattern implementation</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1428,7 +1704,12 @@
           <t>Deep learning, Green AI, Inference, Language models, Model serving</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1446,7 +1727,12 @@
           <t>Behavioral difference, Large language models, Test generation</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1464,7 +1750,12 @@
           <t>Code conversion, Model explainability, Transcoding</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1482,7 +1773,12 @@
           <t>code recommenders, LLM, secure software development, systematic literature review</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1500,7 +1796,12 @@
           <t>Machine learning for software engineering, Software measurement and analytics, Software quality assurance</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1518,7 +1819,12 @@
           <t>Code generation, Language models, Programming tasks</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1536,7 +1842,12 @@
           <t>Automated code synthesis, Machine learning in software development, Natural language programming, Program synthesis, Software engineering automation, Transformer-based models</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1554,7 +1865,12 @@
           <t>AI-assisted software engineering, automated code generation, DevOps automation, Large Language Models (LLMs), software architecture, Software Development Lifecycle (SDLC), software testing</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1572,7 +1888,12 @@
           <t>aggregate computing, code generation, internet of things, Large language models, macroprogramming</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1590,7 +1911,12 @@
           <t>code pre-trained models, Large language models, parameter-efficient fine-tuning, probing analysis</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1608,7 +1934,12 @@
           <t>Conversational interfaces, Conversational low-code development, DSL agent, DSLs, Large Language Models, Vibe coding</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1626,7 +1957,12 @@
           <t>Large Language Models, Program Synthesis, Program Verification, Verus</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1644,7 +1980,12 @@
           <t>automated software testing, large language models, low-rank adaptation codestral mamba model, test case generation</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1662,7 +2003,12 @@
           <t>blockchain, code generation, generative artificial intelligence (Gen-AI), large language models (LLMs), model-driven engineering (MDE), smart contracts, software engineering</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1680,7 +2026,12 @@
           <t>Code translation, Human-centered AI, Large Language Model, Software engineering</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr"/>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1698,7 +2049,12 @@
           <t>Code completion, Code repair, Masked diffusion models, Structured code generation, Syntax-aware masking</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr"/>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1716,7 +2072,12 @@
           <t>AI adoption, Code generation tools, Generative AI, Human-AI interaction</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1734,7 +2095,12 @@
           <t>Code generation, Code semantics, Code understanding, Large language models for code, Program transformation</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1752,7 +2118,12 @@
           <t>Automated program repair, Code Language Models, Large language models, Patch generation, Security vulnerability, Source code</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1770,7 +2141,12 @@
           <t>AI-based code, code generation, software engineering</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1788,7 +2164,12 @@
           <t>code generation, empirical study, large language models, parameter-efficient fine-tuning, quantization, retrieval-augmented generation</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1806,7 +2187,12 @@
           <t>chain of thought, code generation, knowledge distill, large language models</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1824,7 +2210,12 @@
           <t>data mining, machine learning, software engineering</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1842,7 +2233,12 @@
           <t>Bugs, Empirical study, Large language models, Software testing</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1860,7 +2256,12 @@
           <t>Challenges, Large Language Models, LLM4SE</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1878,7 +2279,12 @@
           <t>Data Privacy, Federated Learning, Open Source Code Model, Software Engineering</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr"/>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1896,7 +2302,12 @@
           <t>Code Gen AI in healthcare, code generative AI, large language models, LLM, rich data, self-evolving software, SES, software engineering</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr"/>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1914,7 +2325,12 @@
           <t>Empirical study, Large language models, Literature review, Software engineering</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr"/>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1932,7 +2348,12 @@
           <t>Code Evaluation, Code Generation, Code Pre-trained Language Model</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr"/>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1950,7 +2371,12 @@
           <t>AI assistants, LLMs, Software development lifecycle</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr"/>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1968,7 +2394,12 @@
           <t>code generation, large language model, non-determinism</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr"/>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1986,7 +2417,12 @@
           <t>Design patterns, large language models, pattern application, pattern-based refactoring, quantitative assessment</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2004,7 +2440,12 @@
           <t>bibliometric, content analysis, Large Language Models, LLM, software engineering</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2022,7 +2463,12 @@
           <t>Automated code generation, large language models, software design</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2040,7 +2486,12 @@
           <t>AI-Assisted Programming, Large Language Models, Performance Optimization, Prompt Engineering, Software Development, Structured Prompts</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2058,7 +2509,12 @@
           <t>Clone detection, code duplication, fine-tuning, instruction tuning, large language models, natural language processing, transformers</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2076,7 +2532,12 @@
           <t>Artificial intelligence, ChatGPT, large language model, programming, software development</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2094,7 +2555,12 @@
           <t>artificial intelligence, code generation, data analysis, GenAI4Science, large language models, LLMs4Science, research methods</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2112,7 +2578,12 @@
           <t>code generation, Large language models, prompt programming</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2130,7 +2601,12 @@
           <t>API information, large language model, Project-specific code completion, retrieval-augmented generation</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2144,7 +2620,12 @@
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr"/>
-      <c r="D96" t="inlineStr"/>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2162,7 +2643,12 @@
           <t>automated refactoring, business processes, Microservices extraction, monolith decomposition, natural language processing, performance evaluation, process mining</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2180,7 +2666,12 @@
           <t>Conceptual modeling, Model compiler, Model-driven development, Strategy modeling</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2198,7 +2689,12 @@
           <t>Automated refactoring, code smells, code transformation, deep learning, graph neural networks, object-oriented programming, semantic code modeling, software engineering, software maintenance, software metrics, source code analysis</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr"/>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2216,7 +2712,12 @@
           <t>Code discriminator, code embedding, code generation, code repair</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr"/>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2234,7 +2735,12 @@
           <t>ChatGPT, code generation, Large language model</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr"/>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2252,7 +2758,12 @@
           <t>Code translation, Few-shot learning, Parameter-efficient fine-tuning, Pre-trained language model, Task-adapted prompt tuning</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr"/>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2270,7 +2781,12 @@
           <t>Generative AI, Human-AI interaction, Online communities, Software engineering, Trust</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr"/>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2288,7 +2804,12 @@
           <t>benchmarking, Machine learning for source code, pre-trained models, probing, transformers</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr"/>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2306,7 +2827,12 @@
           <t>Bi-directional LSTM, Code recommendation, Code reuse, Deep learning, GNN, Joint model, LSTM, Recommendation systems, Source code retrieval</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2324,7 +2850,12 @@
           <t>Additional Key Words and PhrasesDeep learning, code generation, language models, Transformer</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr"/>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2342,7 +2873,12 @@
           <t>chain-of-thought, Code generation, large language model, lightweight language model, program language processing</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr"/>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2360,7 +2896,12 @@
           <t>Artificial intelligence, ChatGPT, code quality, code-synthesis, copilot, large language models, model selection</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr"/>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2378,7 +2919,12 @@
           <t>large language model, natural language processing, software development life cycle</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr"/>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2396,7 +2942,12 @@
           <t>natural language processing, software engineering, Test generation</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr"/>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2414,7 +2965,12 @@
           <t>code completion, large language models for code, Membership inference attack, privacy</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2432,7 +2988,12 @@
           <t>AI generated images, Application of AI-powered software, higher education, software engineering, stable diffusion</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr"/>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2450,7 +3011,12 @@
           <t>Code generator, convolutional neural networks, gated recurrent unit, user interface automation</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr"/>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2468,7 +3034,12 @@
           <t>Agile software development, Artificial intelligence, software engineering</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr"/>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2486,7 +3057,12 @@
           <t>Code completion, GitHub copilot, Language model, Testing</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr"/>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2504,7 +3080,12 @@
           <t>code completion, code recommendation, Hierarchical Language Model, language model</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr"/>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2522,7 +3103,12 @@
           <t>Machine learning application, Natural language-based source code generation, Systematic literature review</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr"/>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2540,7 +3126,12 @@
           <t>Naturalistic Programming, Software Engineering, Source Code Generation, Survey</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr"/>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2558,7 +3149,12 @@
           <t>big code, Deep learning, source code generation, source code modeling</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr"/>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2576,7 +3172,12 @@
           <t>deep learning, language model, natural language processing, software engineering, source code</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr"/>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2596,7 +3197,12 @@
           <t>Retrieval Augmented Generation, LangChain, code generation, Vertex AI, FAISS</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2616,7 +3222,12 @@
           <t>RAG, code generation, competitive programming, AST similarity, self-reflection</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr"/>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2636,7 +3247,12 @@
           <t>Retrieval Augmented Generation, Codey APIs, code generation, Vertex AI, RAG</t>
         </is>
       </c>
-      <c r="D123" t="inlineStr"/>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2656,7 +3272,12 @@
           <t>Retrieval-Augmented Code Generation, Repository-Level Code Generation, Survey, Large Language Models, Code Retrieval</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr"/>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2676,7 +3297,12 @@
           <t>L2MAC, large code generation, large language model, von Neumann architecture, external memory</t>
         </is>
       </c>
-      <c r="D125" t="inlineStr"/>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2696,7 +3322,12 @@
           <t>Retrieval-Augmented Generation, code generation, Large Language Models, deterministic retrieval, RAGdeterm</t>
         </is>
       </c>
-      <c r="D126" t="inlineStr"/>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2711,7 +3342,12 @@
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr"/>
-      <c r="D127" t="inlineStr"/>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2731,7 +3367,12 @@
           <t>LangGraph, code generation, RAG, self-correcting agent, diffusers</t>
         </is>
       </c>
-      <c r="D128" t="inlineStr"/>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2751,7 +3392,12 @@
           <t>Retrieval-Augmented Generation, Large Language Models, code generation, SimTalk, embedding models</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr"/>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2771,7 +3417,12 @@
           <t>OWASP LLM Top 10, code generation, prompt injection, static code analysis, AI security</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr"/>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2791,7 +3442,12 @@
           <t>LLMs, code generation, prompt engineering, tokenization, self-consistency</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr"/>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2806,7 +3462,12 @@
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr"/>
-      <c r="D132" t="inlineStr"/>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2826,7 +3487,12 @@
           <t>CodeRAG-Bench, retrieval-augmented generation, code generation, benchmark, retrieval</t>
         </is>
       </c>
-      <c r="D133" t="inlineStr"/>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2846,7 +3512,12 @@
           <t>CodeArena, LLM code generation, collective evaluation, benchmark leakage, evaluation platform</t>
         </is>
       </c>
-      <c r="D134" t="inlineStr"/>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2866,7 +3537,12 @@
           <t>RAG, AST-based chunking, code generation, Tree-sitter, LLM</t>
         </is>
       </c>
-      <c r="D135" t="inlineStr"/>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2886,7 +3562,12 @@
           <t>AI code generation, GitHub Copilot, large language models, code completion, developer productivity</t>
         </is>
       </c>
-      <c r="D136" t="inlineStr"/>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2906,7 +3587,12 @@
           <t>retrieval-augmented generation, control code generation, IEC 61131-3, GPT-4, industrial automation</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr"/>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2922,7 +3608,12 @@
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr"/>
-      <c r="D138" t="inlineStr"/>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2942,7 +3633,12 @@
           <t>AI code generation, agentic workflow, Spring Boot, software construction, human-in-the-loop</t>
         </is>
       </c>
-      <c r="D139" t="inlineStr"/>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2962,7 +3658,12 @@
           <t>generative AI, code completion, GitHub Copilot, ChatGPT, software development</t>
         </is>
       </c>
-      <c r="D140" t="inlineStr"/>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2982,7 +3683,12 @@
           <t>code completion, selective retrieval, RAG, large language model, Repoformer</t>
         </is>
       </c>
-      <c r="D141" t="inlineStr"/>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3002,7 +3708,12 @@
           <t>RAGdeterm, retrieval-augmented generation, code generation, deterministic retrieval, large language models</t>
         </is>
       </c>
-      <c r="D142" t="inlineStr"/>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3022,7 +3733,12 @@
           <t>Code Llama 70B, Mixtral 8x7B, Amazon SageMaker, code generation, large language models</t>
         </is>
       </c>
-      <c r="D143" t="inlineStr"/>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3042,7 +3758,12 @@
           <t>CodeRAG, code generation, code retrieval, graph, large language model</t>
         </is>
       </c>
-      <c r="D144" t="inlineStr"/>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3062,7 +3783,12 @@
           <t>AI-driven code refactoring, legacy code, automatic refactoring, NDC Melbourne, software development</t>
         </is>
       </c>
-      <c r="D145" t="inlineStr"/>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3082,7 +3808,12 @@
           <t>AI code refactoring, software development, large language models, automated refactoring, IBM Bob</t>
         </is>
       </c>
-      <c r="D146" t="inlineStr"/>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3102,7 +3833,12 @@
           <t>agentic refactoring, AI-assisted coding, GitHub Copilot, software engineering productivity, code quality</t>
         </is>
       </c>
-      <c r="D147" t="inlineStr"/>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3122,7 +3858,12 @@
           <t>AI code refactoring, enterprise software modernization, technical debt, best practices, legacy systems</t>
         </is>
       </c>
-      <c r="D148" t="inlineStr"/>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3142,7 +3883,12 @@
           <t>AI coding agents, agentic refactoring, code quality, software engineering, empirical study</t>
         </is>
       </c>
-      <c r="D149" t="inlineStr"/>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3162,7 +3908,12 @@
           <t>AI code refactoring, Augment Code, context engine, best practices, enterprise refactoring</t>
         </is>
       </c>
-      <c r="D150" t="inlineStr"/>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3182,7 +3933,12 @@
           <t>AI Coding Assistant, automated refactoring, technical debt, code quality, CodeScene</t>
         </is>
       </c>
-      <c r="D151" t="inlineStr"/>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3197,7 +3953,12 @@
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr"/>
-      <c r="D152" t="inlineStr"/>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3217,7 +3978,12 @@
           <t>AI refactoring, code quality, CodeScene, automated refactoring, ThoughtWorks podcast</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr"/>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3237,7 +4003,12 @@
           <t>AI-assisted refactoring, generative AI, code maintenance, AI code generation, software development</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr"/>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3257,7 +4028,12 @@
           <t>AI-assisted refactoring, Moderne Platform, OpenRewrite, Lossless Semantic Trees, LLM integration</t>
         </is>
       </c>
-      <c r="D155" t="inlineStr"/>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3277,7 +4053,12 @@
           <t>AI code refactoring, LLMs, language engineering, OpenRewrite, software construction</t>
         </is>
       </c>
-      <c r="D156" t="inlineStr"/>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3297,7 +4078,12 @@
           <t>code refactoring, large language models, empirical study, code quality, prompt engineering</t>
         </is>
       </c>
-      <c r="D157" t="inlineStr"/>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3317,7 +4103,12 @@
           <t>code refactoring, generative AI, Tabnine, AI coding assistant, software development</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr"/>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3337,7 +4128,12 @@
           <t>AI-assisted refactoring, legacy code, Rubberduck, ChatGPT, code transformation</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr"/>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3357,7 +4153,12 @@
           <t>AI code refactoring, LLM limitations, software maintenance, technical debt, developer productivity</t>
         </is>
       </c>
-      <c r="D160" t="inlineStr"/>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3377,7 +4178,12 @@
           <t>code refactoring, large language models, automated software maintenance, hallucination, IDE integration</t>
         </is>
       </c>
-      <c r="D161" t="inlineStr"/>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3397,7 +4203,12 @@
           <t>AI code refactoring, automated refactoring, code quality, developer tools, Graphite</t>
         </is>
       </c>
-      <c r="D162" t="inlineStr"/>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3417,7 +4228,12 @@
           <t>code refactoring, agentic AI, reinforcement learning, large language models, OpenAI Codex</t>
         </is>
       </c>
-      <c r="D163" t="inlineStr"/>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -3437,7 +4253,12 @@
           <t>AI code refactoring, agentic AI, technical debt, software maintenance, guardrails</t>
         </is>
       </c>
-      <c r="D164" t="inlineStr"/>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -3457,7 +4278,12 @@
           <t>AI-driven refactoring, Roslyn analyzers, .NET 9, code mods, automated migration</t>
         </is>
       </c>
-      <c r="D165" t="inlineStr"/>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -3477,7 +4303,12 @@
           <t>code refactoring, ChatGPT, Gemini, Codeium, SonarQube</t>
         </is>
       </c>
-      <c r="D166" t="inlineStr"/>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -3497,7 +4328,12 @@
           <t>AI-assisted refactoring, Rovo Dev, feature flag cleanup, large-scale codebase, code transformation</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr"/>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -3517,7 +4353,12 @@
           <t>Automated code refactoring, AI-powered code transformation, Code modernization, Technical debt reduction, Legacy code migration</t>
         </is>
       </c>
-      <c r="D168" t="inlineStr"/>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -3537,7 +4378,12 @@
           <t>software refactoring, AI tools, ChatGPT, GPT-4, prompt-engineering</t>
         </is>
       </c>
-      <c r="D169" t="inlineStr"/>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -3557,7 +4403,12 @@
           <t>competitive program generation, LLM evaluation, error taxonomy, DeepSeek-R1, benchmark</t>
         </is>
       </c>
-      <c r="D170" t="inlineStr"/>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3577,7 +4428,12 @@
           <t>program synthesis, large language models, fine-tuning, byT5, program-writer</t>
         </is>
       </c>
-      <c r="D171" t="inlineStr"/>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -3597,7 +4453,12 @@
           <t>GenAssist, XR program generation, retrieval-augmented generation, closed-loop feedback, natural language programming</t>
         </is>
       </c>
-      <c r="D172" t="inlineStr"/>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -3617,7 +4478,12 @@
           <t>competitive programming, code generation, large language models, error taxonomy, DeepSeek-R1</t>
         </is>
       </c>
-      <c r="D173" t="inlineStr"/>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -3637,7 +4503,12 @@
           <t>Language Models, Program Generation, Reliability, Explainability, CodeT5</t>
         </is>
       </c>
-      <c r="D174" t="inlineStr"/>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -3657,7 +4528,12 @@
           <t>Program Generation, Large Language Models, Best Practices, Chain of Thought, AI Verification</t>
         </is>
       </c>
-      <c r="D175" t="inlineStr"/>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -3677,7 +4553,12 @@
           <t>tensor programs, language model, deep learning, compilation, code generation</t>
         </is>
       </c>
-      <c r="D176" t="inlineStr"/>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -3697,7 +4578,12 @@
           <t>Large Language Models, System-Level Test, program generation, non-functional properties, Reinforcement Learning</t>
         </is>
       </c>
-      <c r="D177" t="inlineStr"/>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -3713,7 +4599,12 @@
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr"/>
-      <c r="D178" t="inlineStr"/>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3733,7 +4624,12 @@
           <t>Convo, conversational programming language, Generative AI, LLM-based code generation, natural language programming</t>
         </is>
       </c>
-      <c r="D179" t="inlineStr"/>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -3753,7 +4649,12 @@
           <t>Generative AI, test program generation, semiconductor validation, Gherkin test plans, Test and Measurement</t>
         </is>
       </c>
-      <c r="D180" t="inlineStr"/>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -3773,7 +4674,12 @@
           <t>code generation, deep learning, large language models, program synthesis, survey</t>
         </is>
       </c>
-      <c r="D181" t="inlineStr"/>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -3793,7 +4699,12 @@
           <t>Code LLMs, Survey, Software Engineering, Code Generation, NLP</t>
         </is>
       </c>
-      <c r="D182" t="inlineStr"/>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3813,7 +4724,12 @@
           <t>UOFast, VectorShift, UniData, Retrieval-Augmented Generation, legacy system integration</t>
         </is>
       </c>
-      <c r="D183" t="inlineStr"/>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -3833,7 +4749,12 @@
           <t>LLM numerical representations, numerical reasoning, code synthesis, differential testing, LLM4FP</t>
         </is>
       </c>
-      <c r="D184" t="inlineStr"/>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -3853,7 +4774,12 @@
           <t>LLM, code generation, structured generation, neuro-symbolic AI, reinforcement learning</t>
         </is>
       </c>
-      <c r="D185" t="inlineStr"/>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -3868,7 +4794,12 @@
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr"/>
-      <c r="D186" t="inlineStr"/>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -3888,7 +4819,12 @@
           <t>Core War, Digital Red Queen (DRQ), adversarial evolution, large language models, self-play</t>
         </is>
       </c>
-      <c r="D187" t="inlineStr"/>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3908,7 +4844,12 @@
           <t>LLM-driven mutation, program evolution, convergence, structural homogeneity, genetic programming</t>
         </is>
       </c>
-      <c r="D188" t="inlineStr"/>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -3928,7 +4869,12 @@
           <t>program evolution, ShinkaEvolve, sample efficiency, open-ended, AutoML</t>
         </is>
       </c>
-      <c r="D189" t="inlineStr"/>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -3944,7 +4890,12 @@
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr"/>
-      <c r="D190" t="inlineStr"/>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -3964,7 +4915,12 @@
           <t>Applied Generative AI, Agentic AI, Claude Code, Microsoft Copilot, LangChain</t>
         </is>
       </c>
-      <c r="D191" t="inlineStr"/>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -3984,7 +4940,12 @@
           <t>Generative AI, Agentic AI, Claude Code, LLM Application Development, AI Coding</t>
         </is>
       </c>
-      <c r="D192" t="inlineStr"/>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -4004,7 +4965,12 @@
           <t>ShinkaEvolve, program evolution, sample efficiency, large language models, competitive programming</t>
         </is>
       </c>
-      <c r="D193" t="inlineStr"/>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -4024,7 +4990,12 @@
           <t>CoCoEvo, code generation, test case generation, co-evolution, large language models</t>
         </is>
       </c>
-      <c r="D194" t="inlineStr"/>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -4044,7 +5015,12 @@
           <t>generative AI, AI agents, tutorial, software development</t>
         </is>
       </c>
-      <c r="D195" t="inlineStr"/>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -4059,7 +5035,12 @@
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr"/>
-      <c r="D196" t="inlineStr"/>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -4079,7 +5060,12 @@
           <t>code contracts, Design by Contract, generative AI, large language models, JML</t>
         </is>
       </c>
-      <c r="D197" t="inlineStr"/>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -4099,7 +5085,12 @@
           <t>Core War, Digital Red Queen, MAP-Elites, adversarial program evolution, LLM mutation</t>
         </is>
       </c>
-      <c r="D198" t="inlineStr"/>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4119,7 +5110,12 @@
           <t>GEPA, prompt optimization, program evolution, automatic code improvement, DSPy</t>
         </is>
       </c>
-      <c r="D199" t="inlineStr"/>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4139,7 +5135,12 @@
           <t>Coursera specialization, NLP, language models, production API deployment, multimodal AI</t>
         </is>
       </c>
-      <c r="D200" t="inlineStr"/>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4159,7 +5160,12 @@
           <t>Digital Red Queen, DRQ, adversarial program evolution, Core War, LLM</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr"/>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4179,7 +5185,12 @@
           <t>large language models, software engineering, code generation, transformer, cybersecurity</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr"/>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4199,7 +5210,12 @@
           <t>Gen AI Skillup, Google Cloud, generative AI, developer learning path, Gemini</t>
         </is>
       </c>
-      <c r="D203" t="inlineStr"/>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4219,7 +5235,12 @@
           <t>software development, DevOps, API, CI/CD, AI coding tools</t>
         </is>
       </c>
-      <c r="D204" t="inlineStr"/>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4239,7 +5260,12 @@
           <t>code-llm, survey, code-generation, software-engineering, datasets</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr"/>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4259,7 +5285,12 @@
           <t>awesome-list, AI coding tools, code generation, LLMs, software construction</t>
         </is>
       </c>
-      <c r="D206" t="inlineStr"/>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4279,7 +5310,12 @@
           <t>survey, code generation, large language models, LLMs, software engineering</t>
         </is>
       </c>
-      <c r="D207" t="inlineStr"/>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -4299,7 +5335,12 @@
           <t>code generation, fine-tuning, CodeGen, Hugging Face Transformers, LLM</t>
         </is>
       </c>
-      <c r="D208" t="inlineStr"/>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -4319,7 +5360,12 @@
           <t>spec-driven development, Spec Kit, coding agents, AI-assisted coding, software construction</t>
         </is>
       </c>
-      <c r="D209" t="inlineStr"/>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -4339,7 +5385,12 @@
           <t>zed, code editor, rust, collaborative editing, open source</t>
         </is>
       </c>
-      <c r="D210" t="inlineStr"/>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -4359,7 +5410,12 @@
           <t>CodeGeeX, multilingual code generation, code translation, HumanEval-X, large language model</t>
         </is>
       </c>
-      <c r="D211" t="inlineStr"/>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -4379,7 +5435,12 @@
           <t>MiniMax-M2.7, code generation, self-evolution, agent teams, software engineering</t>
         </is>
       </c>
-      <c r="D212" t="inlineStr"/>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -4395,7 +5456,12 @@
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr"/>
-      <c r="D213" t="inlineStr"/>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -4415,7 +5481,12 @@
           <t>Jupyter AI, JupyterLab extension, AI agents, ACP, notebook coding assistant</t>
         </is>
       </c>
-      <c r="D214" t="inlineStr"/>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -4435,7 +5506,12 @@
           <t>GitHub Copilot, GitHub Copilot Chat, Visual Studio Code, code completion, feedback repository</t>
         </is>
       </c>
-      <c r="D215" t="inlineStr"/>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -4455,7 +5531,12 @@
           <t>code completion, IDE plugin, local LLM, IntelliJ IDEA, codellama</t>
         </is>
       </c>
-      <c r="D216" t="inlineStr"/>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -4475,7 +5556,12 @@
           <t>Vue.js, JavaScript framework, web UI, frontend tooling, open-source ecosystem</t>
         </is>
       </c>
-      <c r="D217" t="inlineStr"/>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -4495,7 +5581,12 @@
           <t>GitHub Community, community, open source, discussions</t>
         </is>
       </c>
-      <c r="D218" t="inlineStr"/>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -4515,7 +5606,12 @@
           <t>GitHub Copilot, JetBrains, plugin, code completion, AI coding assistant</t>
         </is>
       </c>
-      <c r="D219" t="inlineStr"/>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -4535,7 +5631,12 @@
           <t>GitHub Copilot, certification, exam outline, AI-assisted coding, prompt engineering</t>
         </is>
       </c>
-      <c r="D220" t="inlineStr"/>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -4555,7 +5656,12 @@
           <t>Developer Experience, AI Coding Tools, Productivity, Collaboration, Survey</t>
         </is>
       </c>
-      <c r="D221" t="inlineStr"/>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -4575,7 +5681,12 @@
           <t>code generation, awesome list, pretrained models, code understanding, datasets</t>
         </is>
       </c>
-      <c r="D222" t="inlineStr"/>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -4595,7 +5706,12 @@
           <t>type-constrained code generation, incremental parsing, language models, TypeScript, constrained sampling</t>
         </is>
       </c>
-      <c r="D223" t="inlineStr"/>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -4615,7 +5731,12 @@
           <t>Copilot4Eclipse, Eclipse, code completion, discussion forum, GitHub Copilot</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr"/>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -4635,7 +5756,12 @@
           <t>CodeJudge, code evaluation, large language models, semantic correctness, test-free evaluation</t>
         </is>
       </c>
-      <c r="D225" t="inlineStr"/>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -4655,7 +5781,12 @@
           <t>automated refactoring, design smell detection, LLM, pull request generation, Checkstyle</t>
         </is>
       </c>
-      <c r="D226" t="inlineStr"/>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -4675,7 +5806,12 @@
           <t>LLM, self-improving software, code evolution, genetic algorithm, multi-agent system</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr"/>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -4695,7 +5831,12 @@
           <t>tree search, PUCT, LLM-guided code evolution, OpenEvolve, code optimization</t>
         </is>
       </c>
-      <c r="D228" t="inlineStr"/>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -4715,7 +5856,12 @@
           <t>RAG, reasoning, retrieval-augmented generation, LLM, survey</t>
         </is>
       </c>
-      <c r="D229" t="inlineStr"/>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -4735,7 +5881,12 @@
           <t>Large Language Models, Software Engineering, Code LLMs, Survey, LLM4SE</t>
         </is>
       </c>
-      <c r="D230" t="inlineStr"/>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -4755,7 +5906,12 @@
           <t>Refact.ai, AI Agent, software construction, SWE-bench, open-source</t>
         </is>
       </c>
-      <c r="D231" t="inlineStr"/>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -4775,7 +5931,12 @@
           <t>openevolve, evolutionary coding agent, LLM-based code optimization, MAP-Elites, genetic algorithm</t>
         </is>
       </c>
-      <c r="D232" t="inlineStr"/>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -4795,7 +5956,12 @@
           <t>Emacs, LLM, library, tool use, coding assistance</t>
         </is>
       </c>
-      <c r="D233" t="inlineStr"/>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -4815,7 +5981,12 @@
           <t>OpenAgents Control, AI agents, code generation, context-aware coding, approval gates</t>
         </is>
       </c>
-      <c r="D234" t="inlineStr"/>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -4835,7 +6006,12 @@
           <t>Codex CLI, coding agent, terminal, software construction, AI coding assistant</t>
         </is>
       </c>
-      <c r="D235" t="inlineStr"/>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -4855,7 +6031,12 @@
           <t>ReforgeAI, Agentic AI, Legacy Modernization, Java Code Refactoring, Framework Migration</t>
         </is>
       </c>
-      <c r="D236" t="inlineStr"/>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -4875,7 +6056,12 @@
           <t>CodeScene, pr-refactoring-agent, code health, refactoring, GitHub Action</t>
         </is>
       </c>
-      <c r="D237" t="inlineStr"/>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -4895,7 +6081,12 @@
           <t>awesome list, AI agents, self-evolution, coding agents, memory systems</t>
         </is>
       </c>
-      <c r="D238" t="inlineStr"/>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -4915,7 +6106,12 @@
           <t>llm-templates, ollama, tabbyapi, code-generation, genai</t>
         </is>
       </c>
-      <c r="D239" t="inlineStr"/>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -4935,7 +6131,12 @@
           <t>Cline, coding agent, IDE extension, autonomous coding, LLM</t>
         </is>
       </c>
-      <c r="D240" t="inlineStr"/>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -4955,7 +6156,12 @@
           <t>AI agent benchmarks, software engineering, coding, function calling, tool use</t>
         </is>
       </c>
-      <c r="D241" t="inlineStr"/>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -4975,7 +6181,12 @@
           <t>Rutex, AI coding agent, Acode plugin, autonomous, mobile development</t>
         </is>
       </c>
-      <c r="D242" t="inlineStr"/>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -4995,7 +6206,12 @@
           <t>llm-loop, autonomous coding agent, LLM CLI plugin, code generation, tool use</t>
         </is>
       </c>
-      <c r="D243" t="inlineStr"/>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -5015,7 +6231,12 @@
           <t>SMELLCC, code smell refactoring, Large Language Model, VS Code extension, SonarLint</t>
         </is>
       </c>
-      <c r="D244" t="inlineStr"/>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -5035,7 +6256,12 @@
           <t>consult-llm, AI second opinion, agent workflow, code review, multi-model debate</t>
         </is>
       </c>
-      <c r="D245" t="inlineStr"/>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -5055,7 +6281,12 @@
           <t>SocialAgent, survey, social simulation, LLM-based agents, resources</t>
         </is>
       </c>
-      <c r="D246" t="inlineStr"/>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -5075,7 +6306,12 @@
           <t>PRO-V, Verilog, RTL Verification, Multi-Agent System, Reinforcement Learning</t>
         </is>
       </c>
-      <c r="D247" t="inlineStr"/>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -5095,7 +6331,12 @@
           <t>ALIA, language model, pre-training, BSC</t>
         </is>
       </c>
-      <c r="D248" t="inlineStr"/>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -5115,7 +6356,12 @@
           <t>Logic-LM, symbolic solver, logical reasoning, large language models, self-refinement</t>
         </is>
       </c>
-      <c r="D249" t="inlineStr"/>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -5135,7 +6381,12 @@
           <t>llama.cpp, LLM inference, C++, GGML, quantization</t>
         </is>
       </c>
-      <c r="D250" t="inlineStr"/>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -5155,7 +6406,12 @@
           <t>AEnvironment, Agentic RL, environment infrastructure, MCP, coding sandbox</t>
         </is>
       </c>
-      <c r="D251" t="inlineStr"/>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -5175,7 +6431,12 @@
           <t>Dafny, LLM, program verification, annotation, DafnySynth</t>
         </is>
       </c>
-      <c r="D252" t="inlineStr"/>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -5195,7 +6456,12 @@
           <t>VisProg, neuro-symbolic, visual reasoning, program generation, GPT-3</t>
         </is>
       </c>
-      <c r="D253" t="inlineStr"/>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -5215,7 +6481,12 @@
           <t>Convo, conversational programming, LLM, pseudocode, code generation</t>
         </is>
       </c>
-      <c r="D254" t="inlineStr"/>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -5235,7 +6506,12 @@
           <t>MAGE, Pro-V, RTL code generation, multi-agent system, RTL verification</t>
         </is>
       </c>
-      <c r="D255" t="inlineStr"/>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -5255,7 +6531,12 @@
           <t>AlphaOPT, optimization program formulation, large language models, self-improving experience library, library learning</t>
         </is>
       </c>
-      <c r="D256" t="inlineStr"/>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -5275,7 +6556,12 @@
           <t>OpenAPI, MCP server, code generation, LangGraph agent, A2A protocol</t>
         </is>
       </c>
-      <c r="D257" t="inlineStr"/>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -5295,7 +6581,12 @@
           <t>CursorCore, AI-assisted programming, code generation, Assistant-Conversation, Programming-Instruct</t>
         </is>
       </c>
-      <c r="D258" t="inlineStr"/>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -5315,7 +6606,12 @@
           <t>sized types, program generation, termination, OCaml, racket</t>
         </is>
       </c>
-      <c r="D259" t="inlineStr"/>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -5335,7 +6631,12 @@
           <t>TitanFuzz, fuzzing, deep learning libraries, large language models, code generation</t>
         </is>
       </c>
-      <c r="D260" t="inlineStr"/>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -5355,7 +6656,12 @@
           <t>ShinkaEvolve, program evolution, code optimization, LLM, evolutionary algorithms</t>
         </is>
       </c>
-      <c r="D261" t="inlineStr"/>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -5375,7 +6681,12 @@
           <t>Digital Red Queen, Core War, LLM-based program evolution, adversarial self-play, code generation</t>
         </is>
       </c>
-      <c r="D262" t="inlineStr"/>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -5395,7 +6706,12 @@
           <t>program evolution, LLM, code generation, TSP, evolutionary algorithms</t>
         </is>
       </c>
-      <c r="D263" t="inlineStr"/>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -5415,7 +6731,12 @@
           <t>multi-agent systems, large language models, software engineering, literature survey, collaboration</t>
         </is>
       </c>
-      <c r="D264" t="inlineStr"/>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -5435,7 +6756,12 @@
           <t>localpilot, GitHub Copilot, local, code completion, on-device</t>
         </is>
       </c>
-      <c r="D265" t="inlineStr"/>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -5455,7 +6781,12 @@
           <t>IBM Full Stack Software Developer, portfolio, full-stack development, Coursera, certifications</t>
         </is>
       </c>
-      <c r="D266" t="inlineStr"/>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -5475,7 +6806,12 @@
           <t>Forage, JP Morgan, virtual experience, data visualization, Perspective</t>
         </is>
       </c>
-      <c r="D267" t="inlineStr"/>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -5493,7 +6829,12 @@
           <t>CodeArena, code generation, collective evaluation, benchmark leakage, LLMs</t>
         </is>
       </c>
-      <c r="D268" t="inlineStr"/>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -5511,7 +6852,12 @@
           <t>QuanBench+, quantum code generation, multi-framework benchmark, feedback-based repair, large language models</t>
         </is>
       </c>
-      <c r="D269" t="inlineStr"/>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -5529,7 +6875,12 @@
           <t>large language models, code generation, multi-agent collaboration, runtime execution debugging, post-training strategies</t>
         </is>
       </c>
-      <c r="D270" t="inlineStr"/>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -5547,7 +6898,12 @@
           <t>PlayEval, PlayCoder, GUI code generation, multi-agent framework, benchmark</t>
         </is>
       </c>
-      <c r="D271" t="inlineStr"/>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -5565,7 +6921,12 @@
           <t>PaperCoder, code generation, machine learning papers, multi-agent system, paper-to-code</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr"/>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -5583,7 +6944,12 @@
           <t>simple self-distillation, code generation, large language model, supervised fine-tuning, token distribution reshaping</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr"/>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -5601,7 +6967,12 @@
           <t>code generation, reinforcement learning, compiler feedback, exploration, fine-grained optimization</t>
         </is>
       </c>
-      <c r="D274" t="inlineStr"/>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -5619,7 +6990,12 @@
           <t>requirement ambiguity, code generation, benchmark, large language models, Orchid</t>
         </is>
       </c>
-      <c r="D275" t="inlineStr"/>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -5637,7 +7013,12 @@
           <t>Think-Anywhere, code generation, reasoning, reinforcement learning, large language models</t>
         </is>
       </c>
-      <c r="D276" t="inlineStr"/>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -5655,7 +7036,12 @@
           <t>MeshCoder, 3D reconstruction, point cloud, program synthesis, large language model</t>
         </is>
       </c>
-      <c r="D277" t="inlineStr"/>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -5673,7 +7059,12 @@
           <t>A.S.E, AI code generation, security evaluation, repository-level, LLMs</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr"/>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -5691,7 +7082,12 @@
           <t>GLLM, G-code generation, CNC machining, Large Language Models, Retrieval-Augmented Generation</t>
         </is>
       </c>
-      <c r="D279" t="inlineStr"/>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -5709,7 +7105,12 @@
           <t>OpenClassGen, class-level code generation, Python classes, LLM evaluation, dataset</t>
         </is>
       </c>
-      <c r="D280" t="inlineStr"/>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -5727,7 +7128,12 @@
           <t>UI-to-Code generation, agentic framework, interactive code, WebVIA, vision-language models</t>
         </is>
       </c>
-      <c r="D281" t="inlineStr"/>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -5745,7 +7151,12 @@
           <t>HDL generation, large language model, fine-tuning, data synthesis, CodeV</t>
         </is>
       </c>
-      <c r="D282" t="inlineStr"/>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -5763,7 +7174,12 @@
           <t>TeXpert, LaTeX code generation, scientific documents, benchmark, large language models</t>
         </is>
       </c>
-      <c r="D283" t="inlineStr"/>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -5781,7 +7197,12 @@
           <t>Pharo, code completion, low-resource programming languages, continued pre-training, fine-tuning</t>
         </is>
       </c>
-      <c r="D284" t="inlineStr"/>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -5799,7 +7220,12 @@
           <t>program synthesis, CODEGEN, JAXFORMER, multi-turn programming, code generation</t>
         </is>
       </c>
-      <c r="D285" t="inlineStr"/>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -5817,7 +7243,12 @@
           <t>CodeElo, competition-level code generation, Elo rating, CodeForces, LLMs</t>
         </is>
       </c>
-      <c r="D286" t="inlineStr"/>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -5835,7 +7266,12 @@
           <t>RRTF, PanGu-Coder2, code generation, large language models</t>
         </is>
       </c>
-      <c r="D287" t="inlineStr"/>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -5853,7 +7289,12 @@
           <t>ScreenCoder, multi-agent framework, UI-to-code generation, UI grounding, reinforcement learning</t>
         </is>
       </c>
-      <c r="D288" t="inlineStr"/>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -5871,7 +7312,12 @@
           <t>jina-code-embeddings, code retrieval, autoregressive backbone, last-token pooling, cross-lingual code similarity</t>
         </is>
       </c>
-      <c r="D289" t="inlineStr"/>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -5889,7 +7335,12 @@
           <t>Retrieval-Augmented Generation, chunking, Abstract Syntax Trees, code generation, structure-aware</t>
         </is>
       </c>
-      <c r="D290" t="inlineStr"/>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -5907,7 +7358,12 @@
           <t>CodeRL, program synthesis, reinforcement learning, code generation, unit tests</t>
         </is>
       </c>
-      <c r="D291" t="inlineStr"/>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -5925,7 +7381,12 @@
           <t>visual code generation, multimodal evaluation, benchmark, LLM-as-Judge, interactive artifacts</t>
         </is>
       </c>
-      <c r="D292" t="inlineStr"/>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -5943,7 +7404,12 @@
           <t>LeetCodeDataset, code generation, reasoning, supervised fine-tuning, contamination-free evaluation</t>
         </is>
       </c>
-      <c r="D293" t="inlineStr"/>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -5961,7 +7427,12 @@
           <t>ReLook, front-end code generation, reinforcement learning, multimodal LLM, visual grounding</t>
         </is>
       </c>
-      <c r="D294" t="inlineStr"/>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -5979,7 +7450,12 @@
           <t>specification autoformalization, Verus-SpecBench, Verus-SpecGym, formal verification, LLM agents</t>
         </is>
       </c>
-      <c r="D295" t="inlineStr"/>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -5997,7 +7473,12 @@
           <t>mHumanEval, multilingual code generation, benchmark, low-resource languages, cross-lingual code generation</t>
         </is>
       </c>
-      <c r="D296" t="inlineStr"/>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -6015,7 +7496,12 @@
           <t>BigCodeArena, code generation, human evaluation, execution environment, benchmark</t>
         </is>
       </c>
-      <c r="D297" t="inlineStr"/>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -6033,7 +7519,12 @@
           <t>Agents4PLC, PLC code generation, code verification, multi-agent system, RAG</t>
         </is>
       </c>
-      <c r="D298" t="inlineStr"/>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -6051,7 +7542,12 @@
           <t>code compression, long context, Large Language Models, Code LLMs, LongCodeZip</t>
         </is>
       </c>
-      <c r="D299" t="inlineStr"/>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -6069,7 +7565,12 @@
           <t>GPIoT, code generation, IoT applications, fine-tuning, small language models</t>
         </is>
       </c>
-      <c r="D300" t="inlineStr"/>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -6087,7 +7588,12 @@
           <t>superoptimization, large language models, reinforcement learning, SuperCoder, assembly generation</t>
         </is>
       </c>
-      <c r="D301" t="inlineStr"/>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -6105,7 +7611,12 @@
           <t>Vibe Coding, large language models, autonomous coding agents, human-AI collaboration, development models</t>
         </is>
       </c>
-      <c r="D302" t="inlineStr"/>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -6123,7 +7634,12 @@
           <t>BEAVER, safety properties, verification, sound bounds, LLM</t>
         </is>
       </c>
-      <c r="D303" t="inlineStr"/>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -6141,7 +7657,12 @@
           <t>SwiftEval, Swift, benchmark, code generation, large language models</t>
         </is>
       </c>
-      <c r="D304" t="inlineStr"/>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -6159,7 +7680,12 @@
           <t>AI agentic programming, coding agents, planning, tool integration, benchmarking</t>
         </is>
       </c>
-      <c r="D305" t="inlineStr"/>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -6177,7 +7703,12 @@
           <t>example-based code generation, large language models, input-output examples, iterative evaluation, code generation benchmark</t>
         </is>
       </c>
-      <c r="D306" t="inlineStr"/>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -6195,7 +7726,12 @@
           <t>CodeFusion, diffusion model, code generation, natural language to code, pre-trained model</t>
         </is>
       </c>
-      <c r="D307" t="inlineStr"/>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr"/>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -6213,7 +7749,12 @@
           <t>Nanbeige4.1-3B, small language model, agentic behavior, code generation, reinforcement learning</t>
         </is>
       </c>
-      <c r="D308" t="inlineStr"/>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -6231,7 +7772,12 @@
           <t>AST-T5, Abstract Syntax Tree, code generation, transpilation, pretraining</t>
         </is>
       </c>
-      <c r="D309" t="inlineStr"/>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -6249,7 +7795,12 @@
           <t>SwallowCode, SwallowMath, program synthesis, mathematical reasoning, data rewriting</t>
         </is>
       </c>
-      <c r="D310" t="inlineStr"/>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -6267,7 +7818,12 @@
           <t>CCTU, LLM tool use, constraint compliance, benchmark evaluation, self-refinement</t>
         </is>
       </c>
-      <c r="D311" t="inlineStr"/>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr"/>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -6285,7 +7841,12 @@
           <t>Long Code Arena, benchmark, code processing, project-level context, code generation</t>
         </is>
       </c>
-      <c r="D312" t="inlineStr"/>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -6303,7 +7864,12 @@
           <t>SALLM, secure code generation, benchmarking, large language models, security</t>
         </is>
       </c>
-      <c r="D313" t="inlineStr"/>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -6321,7 +7887,12 @@
           <t>agentic refactoring, AI coding tools, code quality, refactoring types, empirical study</t>
         </is>
       </c>
-      <c r="D314" t="inlineStr"/>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -6339,7 +7910,12 @@
           <t>Lean Refactor, retrieval-augmented agentic framework, proof refactoring, multi-objective optimization, version robustness</t>
         </is>
       </c>
-      <c r="D315" t="inlineStr"/>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr"/>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -6357,7 +7933,12 @@
           <t>GigaEvo, LLM-guided evolutionary computation, MAP-Elites, AlphaEvolve, quality-diversity</t>
         </is>
       </c>
-      <c r="D316" t="inlineStr"/>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -6375,7 +7956,12 @@
           <t>Claude Code, agentic coding tool, pull request acceptance, software development, empirical study</t>
         </is>
       </c>
-      <c r="D317" t="inlineStr"/>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -6393,7 +7979,12 @@
           <t>GPU kernel optimization, co-evolving world model, K-Search, LLM-guided search, evolutionary search</t>
         </is>
       </c>
-      <c r="D318" t="inlineStr"/>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -6411,7 +8002,12 @@
           <t>Programmatic Skill Network, continual skill acquisition, symbolic programs, large language models, embodied agents</t>
         </is>
       </c>
-      <c r="D319" t="inlineStr"/>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -6429,7 +8025,12 @@
           <t>vibe coding, agentic coding, human-in-the-loop, autonomous software development, hybrid architectures</t>
         </is>
       </c>
-      <c r="D320" t="inlineStr"/>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -6447,7 +8048,12 @@
           <t>code editing, next edit suggestion, dual-model architecture, instruction-free, low-latency</t>
         </is>
       </c>
-      <c r="D321" t="inlineStr"/>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -6462,7 +8068,12 @@
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr"/>
-      <c r="D322" t="inlineStr"/>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -6477,7 +8088,12 @@
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr"/>
-      <c r="D323" t="inlineStr"/>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -6492,7 +8108,12 @@
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr"/>
-      <c r="D324" t="inlineStr"/>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -6510,7 +8131,12 @@
           <t>speculative decoding, draft model training, acceptance rate, LK losses, large language model inference</t>
         </is>
       </c>
-      <c r="D325" t="inlineStr"/>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -6525,7 +8151,12 @@
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr"/>
-      <c r="D326" t="inlineStr"/>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -6540,7 +8171,12 @@
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr"/>
-      <c r="D327" t="inlineStr"/>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -6555,7 +8191,12 @@
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr"/>
-      <c r="D328" t="inlineStr"/>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -6570,7 +8211,12 @@
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr"/>
-      <c r="D329" t="inlineStr"/>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -6585,7 +8231,12 @@
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr"/>
-      <c r="D330" t="inlineStr"/>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -6600,7 +8251,12 @@
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr"/>
-      <c r="D331" t="inlineStr"/>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -6615,7 +8271,12 @@
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr"/>
-      <c r="D332" t="inlineStr"/>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -6630,7 +8291,12 @@
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr"/>
-      <c r="D333" t="inlineStr"/>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -6648,7 +8314,12 @@
           <t>CAD construction sequences, LLM agentic search, program synthesis, vision-language model, parametric CAD dataset</t>
         </is>
       </c>
-      <c r="D334" t="inlineStr"/>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Include</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -6663,7 +8334,12 @@
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr"/>
-      <c r="D335" t="inlineStr"/>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -6681,7 +8357,12 @@
           <t>TikZilla, Text-to-TikZ, reinforcement learning, supervised fine-tuning, DaTikZ-V4</t>
         </is>
       </c>
-      <c r="D336" t="inlineStr"/>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -6696,7 +8377,12 @@
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr"/>
-      <c r="D337" t="inlineStr"/>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -6711,7 +8397,12 @@
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr"/>
-      <c r="D338" t="inlineStr"/>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -6726,7 +8417,12 @@
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr"/>
-      <c r="D339" t="inlineStr"/>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -6741,11 +8437,16 @@
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr"/>
-      <c r="D340" t="inlineStr"/>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Exclude</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E340" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Include,Exclude"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>